<commit_message>
📊 Actualizar PROYECCION_VENTAS_DIA_VU.xlsx — 08-04-2026, 12:08:06 p. m.
</commit_message>
<xml_diff>
--- a/datos/PROYECCION_VENTAS_DIA_VU.xlsx
+++ b/datos/PROYECCION_VENTAS_DIA_VU.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/df502c28020c5b60/Documentos/GIM/Proteccion Familiar/Estrategia/Estrategia 2026/3.Estrategia Comercial 2026/Dash board/Archivos_Base Marzo/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/ABRIL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{50DDB4D2-79BA-4FBA-B32C-3FFEF1A65FA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EC79D71E-5837-437B-B8D9-C9E4254EECFC}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{72962B2A-2139-42D7-98C8-2464BEA22820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A3BE980-EF25-46AD-AB95-C96A15423DF6}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{97D2A031-07BF-4B71-BC0E-1411959519BA}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{97D2A031-07BF-4B71-BC0E-1411959519BA}"/>
   </bookViews>
   <sheets>
     <sheet name="Proyeccion Venta Diaria Q" sheetId="2" r:id="rId1"/>
@@ -65,7 +65,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="164" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -120,9 +120,9 @@
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -131,7 +131,8 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Millares [0]" xfId="2" builtinId="6"/>
@@ -494,23 +495,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6921A9B2-21D4-4B0E-BEC1-20DEACA014A6}">
   <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.46484375" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.44140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="4">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -527,16 +528,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>3.6956290771551811E-2</v>
+        <v>4.3431934664888663E-2</v>
       </c>
       <c r="C3" s="4">
         <f>+$B$1*B3</f>
-        <v>1.182601304689658</v>
+        <v>1.8675731905902124</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -544,471 +545,471 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>7.0730541212468925E-2</v>
+        <v>4.5531629201428545E-2</v>
       </c>
       <c r="C4" s="4">
         <f t="shared" ref="C4:C33" si="0">+$B$1*B4</f>
-        <v>2.2633773187990056</v>
+        <v>1.9578600556614274</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" ref="E4:E33" si="1">+($B$1*(D4*$B$33)/C4)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>0.10384163815335309</v>
+        <v>6.02387488363808E-2</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="0"/>
-        <v>3.322932420907299</v>
+        <v>2.5902661999643746</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>0.13186797473732448</v>
+        <v>7.332770271062157E-2</v>
       </c>
       <c r="C6" s="4">
         <f t="shared" si="0"/>
-        <v>4.2197751915943833</v>
+        <v>3.1530912165567275</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>0.15931174916905069</v>
+        <v>0.10368544944589318</v>
       </c>
       <c r="C7" s="4">
         <f t="shared" si="0"/>
-        <v>5.0979759734096222</v>
+        <v>4.4584743261734072</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>0.17339439912854135</v>
+        <v>9.1318271652995262E-2</v>
       </c>
       <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>5.5486207721133232</v>
+        <v>3.9266856810787965</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9" s="3">
-        <v>0.19953407243133525</v>
+        <v>0.12194818224154563</v>
       </c>
       <c r="C9" s="4">
         <f t="shared" si="0"/>
-        <v>6.3850903178027281</v>
+        <v>5.243771836386462</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
       <c r="B10" s="3">
-        <v>0.21212741552113223</v>
+        <v>0.11438163752027036</v>
       </c>
       <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>6.7880772966762315</v>
+        <v>4.9184104133716255</v>
       </c>
       <c r="E10" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
       <c r="B11" s="3">
-        <v>0.25241833902718575</v>
+        <v>0.1382239569442768</v>
       </c>
       <c r="C11" s="4">
         <f t="shared" si="0"/>
-        <v>8.0773868488699438</v>
+        <v>5.9436301486039023</v>
       </c>
       <c r="E11" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
       <c r="B12" s="3">
-        <v>0.28858519729806292</v>
+        <v>0.17479167443461371</v>
       </c>
       <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>9.2347263135380135</v>
+        <v>7.5160420006883895</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
       <c r="B13" s="3">
-        <v>0.31916094065827749</v>
+        <v>0.17991318751952692</v>
       </c>
       <c r="C13" s="4">
         <f t="shared" si="0"/>
-        <v>10.21315010106488</v>
+        <v>7.7362670633396577</v>
       </c>
       <c r="E13" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
       <c r="B14" s="3">
-        <v>0.3710932431673552</v>
+        <v>0.19294033692563695</v>
       </c>
       <c r="C14" s="4">
         <f t="shared" si="0"/>
-        <v>11.874983781355366</v>
+        <v>8.2964344878023883</v>
       </c>
       <c r="E14" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
       <c r="B15" s="3">
-        <v>0.39655650496602957</v>
+        <v>0.21121725433144362</v>
       </c>
       <c r="C15" s="4">
         <f t="shared" si="0"/>
-        <v>12.689808158912946</v>
+        <v>9.0823419362520763</v>
       </c>
       <c r="E15" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
       <c r="B16" s="3">
-        <v>0.41330376661630752</v>
+        <v>0.21219716981462325</v>
       </c>
       <c r="C16" s="4">
         <f t="shared" si="0"/>
-        <v>13.225720531721841</v>
+        <v>9.1244783020288001</v>
       </c>
       <c r="E16" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>15</v>
       </c>
       <c r="B17" s="3">
-        <v>0.44666423331010763</v>
+        <v>0.23627111850348265</v>
       </c>
       <c r="C17" s="4">
         <f t="shared" si="0"/>
-        <v>14.293255465923444</v>
+        <v>10.159658095649753</v>
       </c>
       <c r="E17" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>0.46168480944179474</v>
+        <v>0.24932669307579572</v>
       </c>
       <c r="C18" s="4">
         <f t="shared" si="0"/>
-        <v>14.773913902137432</v>
+        <v>10.721047802259216</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>17</v>
       </c>
       <c r="B19" s="3">
-        <v>0.50976876296310047</v>
+        <v>0.268747597747724</v>
       </c>
       <c r="C19" s="4">
         <f t="shared" si="0"/>
-        <v>16.312600414819215</v>
+        <v>11.556146703152132</v>
       </c>
       <c r="E19" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>18</v>
       </c>
       <c r="B20" s="3">
-        <v>0.53874801416457396</v>
+        <v>0.2869340810194404</v>
       </c>
       <c r="C20" s="4">
         <f t="shared" si="0"/>
-        <v>17.239936453266367</v>
+        <v>12.338165483835937</v>
       </c>
       <c r="E20" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>0.57354402285616501</v>
+        <v>0.29508994118778675</v>
       </c>
       <c r="C21" s="4">
         <f t="shared" si="0"/>
-        <v>18.35340873139728</v>
+        <v>12.688867471074831</v>
       </c>
       <c r="E21" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>0.590118708404618</v>
+        <v>0.29875621187328866</v>
       </c>
       <c r="C22" s="4">
         <f t="shared" si="0"/>
-        <v>18.883798668947776</v>
+        <v>12.846517110551412</v>
       </c>
       <c r="E22" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>0.61219544963029537</v>
+        <v>0.32643044200553584</v>
       </c>
       <c r="C23" s="4">
         <f t="shared" si="0"/>
-        <v>19.590254388169452</v>
+        <v>14.036509006238042</v>
       </c>
       <c r="E23" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>0.65080290206753511</v>
+        <v>0.34296152497092097</v>
       </c>
       <c r="C24" s="4">
         <f t="shared" si="0"/>
-        <v>20.825692866161123</v>
+        <v>14.747345573749602</v>
       </c>
       <c r="E24" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>0.67591829101271117</v>
+        <v>0.3453528608483149</v>
       </c>
       <c r="C25" s="4">
         <f t="shared" si="0"/>
-        <v>21.629385312406757</v>
+        <v>14.850173016477541</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>0.70496537561535133</v>
+        <v>0.37004276174482909</v>
       </c>
       <c r="C26" s="4">
         <f t="shared" si="0"/>
-        <v>22.558892019691243</v>
+        <v>15.911838755027651</v>
       </c>
       <c r="E26" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>25</v>
       </c>
       <c r="B27" s="3">
-        <v>0.74848013909223288</v>
+        <v>0.39272435790101479</v>
       </c>
       <c r="C27" s="4">
         <f t="shared" si="0"/>
-        <v>23.951364450951452</v>
+        <v>16.887147389743635</v>
       </c>
       <c r="E27" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>26</v>
       </c>
       <c r="B28" s="3">
-        <v>0.7883266528343289</v>
+        <v>0.40340547059461362</v>
       </c>
       <c r="C28" s="4">
         <f t="shared" si="0"/>
-        <v>25.226452890698525</v>
+        <v>17.346435235568386</v>
       </c>
       <c r="E28" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>27</v>
       </c>
       <c r="B29" s="3">
-        <v>0.80291053847691751</v>
+        <v>0.409773198998163</v>
       </c>
       <c r="C29" s="4">
         <f t="shared" si="0"/>
-        <v>25.69313723126136</v>
+        <v>17.620247556921008</v>
       </c>
       <c r="E29" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>28</v>
       </c>
       <c r="B30" s="3">
-        <v>0.83265548488853058</v>
+        <v>0.4385088884701433</v>
       </c>
       <c r="C30" s="4">
         <f t="shared" si="0"/>
-        <v>26.644975516432979</v>
+        <v>18.855882204216162</v>
       </c>
       <c r="E30" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>29</v>
       </c>
       <c r="B31" s="3">
-        <v>0.87651827139422922</v>
+        <v>0.44472863662132905</v>
       </c>
       <c r="C31" s="4">
         <f t="shared" si="0"/>
-        <v>28.048584684615335</v>
+        <v>19.12333137471715</v>
       </c>
       <c r="E31" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>30</v>
       </c>
       <c r="B32" s="3">
-        <v>0.9449023258302931</v>
+        <v>0.49648073777651436</v>
       </c>
       <c r="C32" s="4">
         <f t="shared" si="0"/>
-        <v>30.236874426569379</v>
+        <v>21.348671724390119</v>
       </c>
       <c r="E32" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -1017,7 +1018,7 @@
       </c>
       <c r="C33" s="4">
         <f t="shared" si="0"/>
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="E33" s="4">
         <f t="shared" si="1"/>
@@ -1037,23 +1038,23 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFE9516D-DB2D-4859-B61B-1A68D75109AA}">
   <dimension ref="A1:E33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.19921875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.86328125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.46484375" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.19921875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.88671875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.6640625" style="4" customWidth="1"/>
+    <col min="5" max="5" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>2</v>
       </c>
       <c r="B1" s="4">
-        <v>104000000</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+        <v>142000000</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1070,16 +1071,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>3.6956290771551811E-2</v>
+        <v>4.3431934664888663E-2</v>
       </c>
       <c r="C3" s="4">
         <f>+$B$1*B3</f>
-        <v>3843454.2402413883</v>
+        <v>6167334.7224141899</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -1087,480 +1088,480 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>7.0730541212468925E-2</v>
+        <v>4.5531629201428545E-2</v>
       </c>
       <c r="C4" s="4">
         <f t="shared" ref="C4:C33" si="0">+$B$1*B4</f>
-        <v>7355976.2860967685</v>
+        <v>6465491.3466028534</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" ref="E4:E33" si="1">+($B$1*(D4*$B$33)/C4)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>0.10384163815335309</v>
+        <v>6.02387488363808E-2</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="0"/>
-        <v>10799530.367948722</v>
+        <v>8553902.3347660732</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>0.13186797473732448</v>
+        <v>7.332770271062157E-2</v>
       </c>
       <c r="C6" s="4">
         <f t="shared" si="0"/>
-        <v>13714269.372681746</v>
+        <v>10412533.784908263</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>0.15931174916905069</v>
+        <v>0.10368544944589318</v>
       </c>
       <c r="C7" s="4">
         <f t="shared" si="0"/>
-        <v>16568421.913581273</v>
+        <v>14723333.821316833</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>0.17339439912854135</v>
+        <v>9.1318271652995262E-2</v>
       </c>
       <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>18033017.5093683</v>
+        <v>12967194.574725328</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9" s="3">
-        <v>0.19953407243133525</v>
+        <v>0.12194818224154563</v>
       </c>
       <c r="C9" s="4">
         <f t="shared" si="0"/>
-        <v>20751543.532858867</v>
+        <v>17316641.878299478</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="1">
         <v>8</v>
       </c>
       <c r="B10" s="3">
-        <v>0.21212741552113223</v>
+        <v>0.11438163752027036</v>
       </c>
       <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>22061251.214197751</v>
+        <v>16242192.527878391</v>
       </c>
       <c r="E10" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>9</v>
       </c>
       <c r="B11" s="3">
-        <v>0.25241833902718575</v>
+        <v>0.1382239569442768</v>
       </c>
       <c r="C11" s="4">
         <f t="shared" si="0"/>
-        <v>26251507.258827318</v>
+        <v>19627801.886087306</v>
       </c>
       <c r="E11" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="1">
         <v>10</v>
       </c>
       <c r="B12" s="3">
-        <v>0.28858519729806292</v>
+        <v>0.17479167443461371</v>
       </c>
       <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>30012860.518998545</v>
+        <v>24820417.769715149</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="1">
         <v>11</v>
       </c>
       <c r="B13" s="3">
-        <v>0.31916094065827749</v>
+        <v>0.17991318751952692</v>
       </c>
       <c r="C13" s="4">
         <f t="shared" si="0"/>
-        <v>33192737.828460861</v>
+        <v>25547672.627772823</v>
       </c>
       <c r="E13" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="1">
         <v>12</v>
       </c>
       <c r="B14" s="3">
-        <v>0.3710932431673552</v>
+        <v>0.19294033692563695</v>
       </c>
       <c r="C14" s="4">
         <f t="shared" si="0"/>
-        <v>38593697.289404944</v>
+        <v>27397527.843440447</v>
       </c>
       <c r="E14" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="1">
         <v>13</v>
       </c>
       <c r="B15" s="3">
-        <v>0.39655650496602957</v>
+        <v>0.21121725433144362</v>
       </c>
       <c r="C15" s="4">
         <f t="shared" si="0"/>
-        <v>41241876.516467072</v>
+        <v>29992850.115064994</v>
       </c>
       <c r="E15" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="1">
         <v>14</v>
       </c>
       <c r="B16" s="3">
-        <v>0.41330376661630752</v>
+        <v>0.21219716981462325</v>
       </c>
       <c r="C16" s="4">
         <f t="shared" si="0"/>
-        <v>42983591.728095986</v>
+        <v>30131998.1136765</v>
       </c>
       <c r="E16" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="1">
         <v>15</v>
       </c>
       <c r="B17" s="3">
-        <v>0.44666423331010763</v>
+        <v>0.23627111850348265</v>
       </c>
       <c r="C17" s="4">
         <f t="shared" si="0"/>
-        <v>46453080.264251195</v>
+        <v>33550498.827494536</v>
       </c>
       <c r="E17" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="1">
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>0.46168480944179474</v>
+        <v>0.24932669307579572</v>
       </c>
       <c r="C18" s="4">
         <f t="shared" si="0"/>
-        <v>48015220.18194665</v>
+        <v>35404390.416762993</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="1">
         <v>17</v>
       </c>
       <c r="B19" s="3">
-        <v>0.50976876296310047</v>
+        <v>0.268747597747724</v>
       </c>
       <c r="C19" s="4">
         <f t="shared" si="0"/>
-        <v>53015951.34816245</v>
+        <v>38162158.880176805</v>
       </c>
       <c r="E19" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="1">
         <v>18</v>
       </c>
       <c r="B20" s="3">
-        <v>0.53874801416457396</v>
+        <v>0.2869340810194404</v>
       </c>
       <c r="C20" s="4">
         <f t="shared" si="0"/>
-        <v>56029793.47311569</v>
+        <v>40744639.504760534</v>
       </c>
       <c r="E20" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="1">
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>0.57354402285616501</v>
+        <v>0.29508994118778675</v>
       </c>
       <c r="C21" s="4">
         <f t="shared" si="0"/>
-        <v>59648578.377041161</v>
+        <v>41902771.648665719</v>
       </c>
       <c r="E21" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="1">
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>0.590118708404618</v>
+        <v>0.29875621187328866</v>
       </c>
       <c r="C22" s="4">
         <f t="shared" si="0"/>
-        <v>61372345.674080275</v>
+        <v>42423382.086006992</v>
       </c>
       <c r="E22" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="1">
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>0.61219544963029537</v>
+        <v>0.32643044200553584</v>
       </c>
       <c r="C23" s="4">
         <f t="shared" si="0"/>
-        <v>63668326.761550717</v>
+        <v>46353122.764786087</v>
       </c>
       <c r="E23" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="1">
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>0.65080290206753511</v>
+        <v>0.34296152497092097</v>
       </c>
       <c r="C24" s="4">
         <f t="shared" si="0"/>
-        <v>67683501.815023646</v>
+        <v>48700536.545870781</v>
       </c>
       <c r="E24" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="1">
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>0.67591829101271117</v>
+        <v>0.3453528608483149</v>
       </c>
       <c r="C25" s="4">
         <f t="shared" si="0"/>
-        <v>70295502.265321955</v>
+        <v>49040106.240460716</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="1">
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>0.70496537561535133</v>
+        <v>0.37004276174482909</v>
       </c>
       <c r="C26" s="4">
         <f t="shared" si="0"/>
-        <v>73316399.063996539</v>
+        <v>52546072.167765729</v>
       </c>
       <c r="E26" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="1">
         <v>25</v>
       </c>
       <c r="B27" s="3">
-        <v>0.74848013909223288</v>
+        <v>0.39272435790101479</v>
       </c>
       <c r="C27" s="4">
         <f t="shared" si="0"/>
-        <v>77841934.46559222</v>
+        <v>55766858.821944103</v>
       </c>
       <c r="E27" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="1">
         <v>26</v>
       </c>
       <c r="B28" s="3">
-        <v>0.7883266528343289</v>
+        <v>0.40340547059461362</v>
       </c>
       <c r="C28" s="4">
         <f t="shared" si="0"/>
-        <v>81985971.894770205</v>
+        <v>57283576.824435137</v>
       </c>
       <c r="E28" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>27</v>
       </c>
       <c r="B29" s="3">
-        <v>0.80291053847691751</v>
+        <v>0.409773198998163</v>
       </c>
       <c r="C29" s="4">
         <f t="shared" si="0"/>
-        <v>83502696.001599416</v>
+        <v>58187794.257739149</v>
       </c>
       <c r="E29" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>28</v>
       </c>
       <c r="B30" s="3">
-        <v>0.83265548488853058</v>
+        <v>0.4385088884701433</v>
       </c>
       <c r="C30" s="4">
         <f t="shared" si="0"/>
-        <v>86596170.428407177</v>
+        <v>62268262.162760347</v>
       </c>
       <c r="E30" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="1">
         <v>29</v>
       </c>
       <c r="B31" s="3">
-        <v>0.87651827139422922</v>
+        <v>0.44472863662132905</v>
       </c>
       <c r="C31" s="4">
         <f t="shared" si="0"/>
-        <v>91157900.224999845</v>
+        <v>63151466.400228724</v>
       </c>
       <c r="E31" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="1">
         <v>30</v>
       </c>
       <c r="B32" s="3">
-        <v>0.9449023258302931</v>
+        <v>0.49648073777651436</v>
       </c>
       <c r="C32" s="4">
         <f t="shared" si="0"/>
-        <v>98269841.886350483</v>
+        <v>70500264.764265046</v>
       </c>
       <c r="E32" s="4">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B33" s="5">
         <v>1</v>
       </c>
       <c r="C33" s="4">
         <f t="shared" si="0"/>
-        <v>104000000</v>
+        <v>142000000</v>
       </c>
       <c r="E33" s="4">
         <f t="shared" si="1"/>

</xml_diff>

<commit_message>
📊 Actualizar PROYECCION_VENTAS_DIA_VU.xlsx — 14-04-2026, 2:12:33 p. m.
</commit_message>
<xml_diff>
--- a/datos/PROYECCION_VENTAS_DIA_VU.xlsx
+++ b/datos/PROYECCION_VENTAS_DIA_VU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos de Mes/ABRIL/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="8_{72962B2A-2139-42D7-98C8-2464BEA22820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5A3BE980-EF25-46AD-AB95-C96A15423DF6}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{72962B2A-2139-42D7-98C8-2464BEA22820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E1DD9CC-A546-40C8-926B-C06D37D267FB}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{97D2A031-07BF-4B71-BC0E-1411959519BA}"/>
   </bookViews>
@@ -532,12 +532,12 @@
       <c r="A3" s="1">
         <v>1</v>
       </c>
-      <c r="B3" s="3">
-        <v>4.3431934664888663E-2</v>
+      <c r="B3" s="5">
+        <v>2.6170453078083591E-2</v>
       </c>
       <c r="C3" s="4">
         <f>+$B$1*B3</f>
-        <v>1.8675731905902124</v>
+        <v>1.1253294823575943</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -549,12 +549,12 @@
       <c r="A4" s="1">
         <v>2</v>
       </c>
-      <c r="B4" s="3">
-        <v>4.5531629201428545E-2</v>
+      <c r="B4" s="5">
+        <v>4.6903732144696002E-2</v>
       </c>
       <c r="C4" s="4">
         <f t="shared" ref="C4:C33" si="0">+$B$1*B4</f>
-        <v>1.9578600556614274</v>
+        <v>2.016860482221928</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" ref="E4:E33" si="1">+($B$1*(D4*$B$33)/C4)</f>
@@ -565,12 +565,12 @@
       <c r="A5" s="1">
         <v>3</v>
       </c>
-      <c r="B5" s="3">
-        <v>6.02387488363808E-2</v>
+      <c r="B5" s="5">
+        <v>7.1151588307445779E-2</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="0"/>
-        <v>2.5902661999643746</v>
+        <v>3.0595182972201687</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="1"/>
@@ -581,12 +581,12 @@
       <c r="A6" s="1">
         <v>4</v>
       </c>
-      <c r="B6" s="3">
-        <v>7.332770271062157E-2</v>
+      <c r="B6" s="5">
+        <v>6.9780141214816085E-2</v>
       </c>
       <c r="C6" s="4">
         <f t="shared" si="0"/>
-        <v>3.1530912165567275</v>
+        <v>3.0005460722370918</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="1"/>
@@ -597,12 +597,12 @@
       <c r="A7" s="1">
         <v>5</v>
       </c>
-      <c r="B7" s="3">
-        <v>0.10368544944589318</v>
+      <c r="B7" s="5">
+        <v>9.5040489969140732E-2</v>
       </c>
       <c r="C7" s="4">
         <f t="shared" si="0"/>
-        <v>4.4584743261734072</v>
+        <v>4.0867410686730512</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="1"/>
@@ -613,12 +613,12 @@
       <c r="A8" s="1">
         <v>6</v>
       </c>
-      <c r="B8" s="3">
-        <v>9.1318271652995262E-2</v>
+      <c r="B8" s="5">
+        <v>0.10977412264119375</v>
       </c>
       <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>3.9266856810787965</v>
+        <v>4.7202872735713317</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="1"/>
@@ -629,12 +629,12 @@
       <c r="A9" s="1">
         <v>7</v>
       </c>
-      <c r="B9" s="3">
-        <v>0.12194818224154563</v>
+      <c r="B9" s="5">
+        <v>0.11899780544643686</v>
       </c>
       <c r="C9" s="4">
         <f t="shared" si="0"/>
-        <v>5.243771836386462</v>
+        <v>5.1169056341967849</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="1"/>
@@ -645,12 +645,12 @@
       <c r="A10" s="1">
         <v>8</v>
       </c>
-      <c r="B10" s="3">
-        <v>0.11438163752027036</v>
+      <c r="B10" s="5">
+        <v>0.12529447699133534</v>
       </c>
       <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>4.9184104133716255</v>
+        <v>5.3876625106274192</v>
       </c>
       <c r="E10" s="4">
         <f t="shared" si="1"/>
@@ -661,12 +661,12 @@
       <c r="A11" s="1">
         <v>9</v>
       </c>
-      <c r="B11" s="3">
-        <v>0.1382239569442768</v>
+      <c r="B11" s="5">
+        <v>0.14159378489820826</v>
       </c>
       <c r="C11" s="4">
         <f t="shared" si="0"/>
-        <v>5.9436301486039023</v>
+        <v>6.0885327506229547</v>
       </c>
       <c r="E11" s="4">
         <f t="shared" si="1"/>
@@ -677,12 +677,12 @@
       <c r="A12" s="1">
         <v>10</v>
       </c>
-      <c r="B12" s="3">
-        <v>0.17479167443461371</v>
+      <c r="B12" s="5">
+        <v>0.17506182941826223</v>
       </c>
       <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>7.5160420006883895</v>
+        <v>7.5276586649852764</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" si="1"/>
@@ -693,12 +693,12 @@
       <c r="A13" s="1">
         <v>11</v>
       </c>
-      <c r="B13" s="3">
-        <v>0.17991318751952692</v>
+      <c r="B13" s="5">
+        <v>0.16342662417529258</v>
       </c>
       <c r="C13" s="4">
         <f t="shared" si="0"/>
-        <v>7.7362670633396577</v>
+        <v>7.027344839537581</v>
       </c>
       <c r="E13" s="4">
         <f t="shared" si="1"/>
@@ -709,12 +709,12 @@
       <c r="A14" s="1">
         <v>12</v>
       </c>
-      <c r="B14" s="3">
-        <v>0.19294033692563695</v>
+      <c r="B14" s="5">
+        <v>0.19708508312213913</v>
       </c>
       <c r="C14" s="4">
         <f t="shared" si="0"/>
-        <v>8.2964344878023883</v>
+        <v>8.4746585742519827</v>
       </c>
       <c r="E14" s="4">
         <f t="shared" si="1"/>
@@ -725,12 +725,12 @@
       <c r="A15" s="1">
         <v>13</v>
       </c>
-      <c r="B15" s="3">
-        <v>0.21121725433144362</v>
+      <c r="B15" s="5">
+        <v>0.22520132940609172</v>
       </c>
       <c r="C15" s="4">
         <f t="shared" si="0"/>
-        <v>9.0823419362520763</v>
+        <v>9.6836571644619447</v>
       </c>
       <c r="E15" s="4">
         <f t="shared" si="1"/>
@@ -741,12 +741,12 @@
       <c r="A16" s="1">
         <v>14</v>
       </c>
-      <c r="B16" s="3">
-        <v>0.21219716981462325</v>
+      <c r="B16" s="5">
+        <v>0.22203649869276915</v>
       </c>
       <c r="C16" s="4">
         <f t="shared" si="0"/>
-        <v>9.1244783020288001</v>
+        <v>9.5475694437890741</v>
       </c>
       <c r="E16" s="4">
         <f t="shared" si="1"/>
@@ -757,12 +757,12 @@
       <c r="A17" s="1">
         <v>15</v>
       </c>
-      <c r="B17" s="3">
-        <v>0.23627111850348265</v>
+      <c r="B17" s="5">
+        <v>0.2387167320396692</v>
       </c>
       <c r="C17" s="4">
         <f t="shared" si="0"/>
-        <v>10.159658095649753</v>
+        <v>10.264819477705776</v>
       </c>
       <c r="E17" s="4">
         <f t="shared" si="1"/>
@@ -773,12 +773,12 @@
       <c r="A18" s="1">
         <v>16</v>
       </c>
-      <c r="B18" s="3">
-        <v>0.24932669307579572</v>
+      <c r="B18" s="5">
+        <v>0.25391932779782045</v>
       </c>
       <c r="C18" s="4">
         <f t="shared" si="0"/>
-        <v>10.721047802259216</v>
+        <v>10.91853109530628</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="1"/>
@@ -789,12 +789,12 @@
       <c r="A19" s="1">
         <v>17</v>
       </c>
-      <c r="B19" s="3">
-        <v>0.268747597747724</v>
+      <c r="B19" s="5">
+        <v>0.25873053532770407</v>
       </c>
       <c r="C19" s="4">
         <f t="shared" si="0"/>
-        <v>11.556146703152132</v>
+        <v>11.125413019091274</v>
       </c>
       <c r="E19" s="4">
         <f t="shared" si="1"/>
@@ -805,12 +805,12 @@
       <c r="A20" s="1">
         <v>18</v>
       </c>
-      <c r="B20" s="3">
-        <v>0.2869340810194404</v>
+      <c r="B20" s="5">
+        <v>0.27706631477459465</v>
       </c>
       <c r="C20" s="4">
         <f t="shared" si="0"/>
-        <v>12.338165483835937</v>
+        <v>11.91385153530757</v>
       </c>
       <c r="E20" s="4">
         <f t="shared" si="1"/>
@@ -821,12 +821,12 @@
       <c r="A21" s="1">
         <v>19</v>
       </c>
-      <c r="B21" s="3">
-        <v>0.29508994118778675</v>
+      <c r="B21" s="5">
+        <v>0.30215662681269789</v>
       </c>
       <c r="C21" s="4">
         <f t="shared" si="0"/>
-        <v>12.688867471074831</v>
+        <v>12.992734952946009</v>
       </c>
       <c r="E21" s="4">
         <f t="shared" si="1"/>
@@ -837,12 +837,12 @@
       <c r="A22" s="1">
         <v>20</v>
       </c>
-      <c r="B22" s="3">
-        <v>0.29875621187328866</v>
+      <c r="B22" s="5">
+        <v>0.32198243112538594</v>
       </c>
       <c r="C22" s="4">
         <f t="shared" si="0"/>
-        <v>12.846517110551412</v>
+        <v>13.845244538391595</v>
       </c>
       <c r="E22" s="4">
         <f t="shared" si="1"/>
@@ -853,12 +853,12 @@
       <c r="A23" s="1">
         <v>21</v>
       </c>
-      <c r="B23" s="3">
-        <v>0.32643044200553584</v>
+      <c r="B23" s="5">
+        <v>0.33302080173822463</v>
       </c>
       <c r="C23" s="4">
         <f t="shared" si="0"/>
-        <v>14.036509006238042</v>
+        <v>14.319894474743659</v>
       </c>
       <c r="E23" s="4">
         <f t="shared" si="1"/>
@@ -869,12 +869,12 @@
       <c r="A24" s="1">
         <v>22</v>
       </c>
-      <c r="B24" s="3">
-        <v>0.34296152497092097</v>
+      <c r="B24" s="5">
+        <v>0.34078606641838294</v>
       </c>
       <c r="C24" s="4">
         <f t="shared" si="0"/>
-        <v>14.747345573749602</v>
+        <v>14.653800855990466</v>
       </c>
       <c r="E24" s="4">
         <f t="shared" si="1"/>
@@ -885,12 +885,12 @@
       <c r="A25" s="1">
         <v>23</v>
       </c>
-      <c r="B25" s="3">
-        <v>0.3453528608483149</v>
+      <c r="B25" s="5">
+        <v>0.34565145319866331</v>
       </c>
       <c r="C25" s="4">
         <f t="shared" si="0"/>
-        <v>14.850173016477541</v>
+        <v>14.863012487542521</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="1"/>
@@ -901,12 +901,12 @@
       <c r="A26" s="1">
         <v>24</v>
       </c>
-      <c r="B26" s="3">
-        <v>0.37004276174482909</v>
+      <c r="B26" s="5">
+        <v>0.36402114934613722</v>
       </c>
       <c r="C26" s="4">
         <f t="shared" si="0"/>
-        <v>15.911838755027651</v>
+        <v>15.6529094218839</v>
       </c>
       <c r="E26" s="4">
         <f t="shared" si="1"/>
@@ -917,12 +917,12 @@
       <c r="A27" s="1">
         <v>25</v>
       </c>
-      <c r="B27" s="3">
-        <v>0.39272435790101479</v>
+      <c r="B27" s="5">
+        <v>0.38577853108457799</v>
       </c>
       <c r="C27" s="4">
         <f t="shared" si="0"/>
-        <v>16.887147389743635</v>
+        <v>16.588476836636854</v>
       </c>
       <c r="E27" s="4">
         <f t="shared" si="1"/>
@@ -933,12 +933,12 @@
       <c r="A28" s="1">
         <v>26</v>
       </c>
-      <c r="B28" s="3">
-        <v>0.40340547059461362</v>
+      <c r="B28" s="5">
+        <v>0.41724024949408756</v>
       </c>
       <c r="C28" s="4">
         <f t="shared" si="0"/>
-        <v>17.346435235568386</v>
+        <v>17.941330728245767</v>
       </c>
       <c r="E28" s="4">
         <f t="shared" si="1"/>
@@ -949,12 +949,12 @@
       <c r="A29" s="1">
         <v>27</v>
       </c>
-      <c r="B29" s="3">
-        <v>0.409773198998163</v>
+      <c r="B29" s="5">
+        <v>0.42837834616153569</v>
       </c>
       <c r="C29" s="4">
         <f t="shared" si="0"/>
-        <v>17.620247556921008</v>
+        <v>18.420268884946037</v>
       </c>
       <c r="E29" s="4">
         <f t="shared" si="1"/>
@@ -965,12 +965,12 @@
       <c r="A30" s="1">
         <v>28</v>
       </c>
-      <c r="B30" s="3">
-        <v>0.4385088884701433</v>
+      <c r="B30" s="5">
+        <v>0.43171235782888068</v>
       </c>
       <c r="C30" s="4">
         <f t="shared" si="0"/>
-        <v>18.855882204216162</v>
+        <v>18.56363138664187</v>
       </c>
       <c r="E30" s="4">
         <f t="shared" si="1"/>
@@ -981,12 +981,12 @@
       <c r="A31" s="1">
         <v>29</v>
       </c>
-      <c r="B31" s="3">
-        <v>0.44472863662132905</v>
+      <c r="B31" s="5">
+        <v>0.46518221262019155</v>
       </c>
       <c r="C31" s="4">
         <f t="shared" si="0"/>
-        <v>19.12333137471715</v>
+        <v>20.002835142668236</v>
       </c>
       <c r="E31" s="4">
         <f t="shared" si="1"/>
@@ -997,12 +997,12 @@
       <c r="A32" s="1">
         <v>30</v>
       </c>
-      <c r="B32" s="3">
-        <v>0.49648073777651436</v>
+      <c r="B32" s="5">
+        <v>0.49168193214591577</v>
       </c>
       <c r="C32" s="4">
         <f t="shared" si="0"/>
-        <v>21.348671724390119</v>
+        <v>21.142323082274377</v>
       </c>
       <c r="E32" s="4">
         <f t="shared" si="1"/>
@@ -1013,7 +1013,7 @@
       <c r="A33" s="1">
         <v>31</v>
       </c>
-      <c r="B33" s="3">
+      <c r="B33" s="5">
         <v>1</v>
       </c>
       <c r="C33" s="4">
@@ -1076,11 +1076,11 @@
         <v>1</v>
       </c>
       <c r="B3" s="3">
-        <v>4.3431934664888663E-2</v>
+        <v>2.6170453078083591E-2</v>
       </c>
       <c r="C3" s="4">
         <f>+$B$1*B3</f>
-        <v>6167334.7224141899</v>
+        <v>3716204.3370878701</v>
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="4">
@@ -1093,11 +1093,11 @@
         <v>2</v>
       </c>
       <c r="B4" s="3">
-        <v>4.5531629201428545E-2</v>
+        <v>4.6903732144696002E-2</v>
       </c>
       <c r="C4" s="4">
         <f t="shared" ref="C4:C33" si="0">+$B$1*B4</f>
-        <v>6465491.3466028534</v>
+        <v>6660329.9645468323</v>
       </c>
       <c r="E4" s="4">
         <f t="shared" ref="E4:E33" si="1">+($B$1*(D4*$B$33)/C4)</f>
@@ -1109,11 +1109,11 @@
         <v>3</v>
       </c>
       <c r="B5" s="3">
-        <v>6.02387488363808E-2</v>
+        <v>7.1151588307445779E-2</v>
       </c>
       <c r="C5" s="4">
         <f t="shared" si="0"/>
-        <v>8553902.3347660732</v>
+        <v>10103525.5396573</v>
       </c>
       <c r="E5" s="4">
         <f t="shared" si="1"/>
@@ -1125,11 +1125,11 @@
         <v>4</v>
       </c>
       <c r="B6" s="3">
-        <v>7.332770271062157E-2</v>
+        <v>6.9780141214816085E-2</v>
       </c>
       <c r="C6" s="4">
         <f t="shared" si="0"/>
-        <v>10412533.784908263</v>
+        <v>9908780.0525038838</v>
       </c>
       <c r="E6" s="4">
         <f t="shared" si="1"/>
@@ -1141,11 +1141,11 @@
         <v>5</v>
       </c>
       <c r="B7" s="3">
-        <v>0.10368544944589318</v>
+        <v>9.5040489969140732E-2</v>
       </c>
       <c r="C7" s="4">
         <f t="shared" si="0"/>
-        <v>14723333.821316833</v>
+        <v>13495749.575617984</v>
       </c>
       <c r="E7" s="4">
         <f t="shared" si="1"/>
@@ -1157,11 +1157,11 @@
         <v>6</v>
       </c>
       <c r="B8" s="3">
-        <v>9.1318271652995262E-2</v>
+        <v>0.10977412264119375</v>
       </c>
       <c r="C8" s="4">
         <f t="shared" si="0"/>
-        <v>12967194.574725328</v>
+        <v>15587925.415049514</v>
       </c>
       <c r="E8" s="4">
         <f t="shared" si="1"/>
@@ -1173,11 +1173,11 @@
         <v>7</v>
       </c>
       <c r="B9" s="3">
-        <v>0.12194818224154563</v>
+        <v>0.11899780544643686</v>
       </c>
       <c r="C9" s="4">
         <f t="shared" si="0"/>
-        <v>17316641.878299478</v>
+        <v>16897688.373394035</v>
       </c>
       <c r="E9" s="4">
         <f t="shared" si="1"/>
@@ -1189,11 +1189,11 @@
         <v>8</v>
       </c>
       <c r="B10" s="3">
-        <v>0.11438163752027036</v>
+        <v>0.12529447699133534</v>
       </c>
       <c r="C10" s="4">
         <f t="shared" si="0"/>
-        <v>16242192.527878391</v>
+        <v>17791815.732769616</v>
       </c>
       <c r="E10" s="4">
         <f t="shared" si="1"/>
@@ -1205,11 +1205,11 @@
         <v>9</v>
       </c>
       <c r="B11" s="3">
-        <v>0.1382239569442768</v>
+        <v>0.14159378489820826</v>
       </c>
       <c r="C11" s="4">
         <f t="shared" si="0"/>
-        <v>19627801.886087306</v>
+        <v>20106317.455545574</v>
       </c>
       <c r="E11" s="4">
         <f t="shared" si="1"/>
@@ -1221,11 +1221,11 @@
         <v>10</v>
       </c>
       <c r="B12" s="3">
-        <v>0.17479167443461371</v>
+        <v>0.17506182941826223</v>
       </c>
       <c r="C12" s="4">
         <f t="shared" si="0"/>
-        <v>24820417.769715149</v>
+        <v>24858779.777393237</v>
       </c>
       <c r="E12" s="4">
         <f t="shared" si="1"/>
@@ -1237,11 +1237,11 @@
         <v>11</v>
       </c>
       <c r="B13" s="3">
-        <v>0.17991318751952692</v>
+        <v>0.16342662417529258</v>
       </c>
       <c r="C13" s="4">
         <f t="shared" si="0"/>
-        <v>25547672.627772823</v>
+        <v>23206580.632891547</v>
       </c>
       <c r="E13" s="4">
         <f t="shared" si="1"/>
@@ -1253,11 +1253,11 @@
         <v>12</v>
       </c>
       <c r="B14" s="3">
-        <v>0.19294033692563695</v>
+        <v>0.19708508312213913</v>
       </c>
       <c r="C14" s="4">
         <f t="shared" si="0"/>
-        <v>27397527.843440447</v>
+        <v>27986081.803343754</v>
       </c>
       <c r="E14" s="4">
         <f t="shared" si="1"/>
@@ -1269,11 +1269,11 @@
         <v>13</v>
       </c>
       <c r="B15" s="3">
-        <v>0.21121725433144362</v>
+        <v>0.22520132940609172</v>
       </c>
       <c r="C15" s="4">
         <f t="shared" si="0"/>
-        <v>29992850.115064994</v>
+        <v>31978588.775665026</v>
       </c>
       <c r="E15" s="4">
         <f t="shared" si="1"/>
@@ -1285,11 +1285,11 @@
         <v>14</v>
       </c>
       <c r="B16" s="3">
-        <v>0.21219716981462325</v>
+        <v>0.22203649869276915</v>
       </c>
       <c r="C16" s="4">
         <f t="shared" si="0"/>
-        <v>30131998.1136765</v>
+        <v>31529182.814373218</v>
       </c>
       <c r="E16" s="4">
         <f t="shared" si="1"/>
@@ -1301,11 +1301,11 @@
         <v>15</v>
       </c>
       <c r="B17" s="3">
-        <v>0.23627111850348265</v>
+        <v>0.2387167320396692</v>
       </c>
       <c r="C17" s="4">
         <f t="shared" si="0"/>
-        <v>33550498.827494536</v>
+        <v>33897775.949633025</v>
       </c>
       <c r="E17" s="4">
         <f t="shared" si="1"/>
@@ -1317,11 +1317,11 @@
         <v>16</v>
       </c>
       <c r="B18" s="3">
-        <v>0.24932669307579572</v>
+        <v>0.25391932779782045</v>
       </c>
       <c r="C18" s="4">
         <f t="shared" si="0"/>
-        <v>35404390.416762993</v>
+        <v>36056544.547290504</v>
       </c>
       <c r="E18" s="4">
         <f t="shared" si="1"/>
@@ -1333,11 +1333,11 @@
         <v>17</v>
       </c>
       <c r="B19" s="3">
-        <v>0.268747597747724</v>
+        <v>0.25873053532770407</v>
       </c>
       <c r="C19" s="4">
         <f t="shared" si="0"/>
-        <v>38162158.880176805</v>
+        <v>36739736.016533978</v>
       </c>
       <c r="E19" s="4">
         <f t="shared" si="1"/>
@@ -1349,11 +1349,11 @@
         <v>18</v>
       </c>
       <c r="B20" s="3">
-        <v>0.2869340810194404</v>
+        <v>0.27706631477459465</v>
       </c>
       <c r="C20" s="4">
         <f t="shared" si="0"/>
-        <v>40744639.504760534</v>
+        <v>39343416.697992437</v>
       </c>
       <c r="E20" s="4">
         <f t="shared" si="1"/>
@@ -1365,11 +1365,11 @@
         <v>19</v>
       </c>
       <c r="B21" s="3">
-        <v>0.29508994118778675</v>
+        <v>0.30215662681269789</v>
       </c>
       <c r="C21" s="4">
         <f t="shared" si="0"/>
-        <v>41902771.648665719</v>
+        <v>42906241.007403098</v>
       </c>
       <c r="E21" s="4">
         <f t="shared" si="1"/>
@@ -1381,11 +1381,11 @@
         <v>20</v>
       </c>
       <c r="B22" s="3">
-        <v>0.29875621187328866</v>
+        <v>0.32198243112538594</v>
       </c>
       <c r="C22" s="4">
         <f t="shared" si="0"/>
-        <v>42423382.086006992</v>
+        <v>45721505.219804801</v>
       </c>
       <c r="E22" s="4">
         <f t="shared" si="1"/>
@@ -1397,11 +1397,11 @@
         <v>21</v>
       </c>
       <c r="B23" s="3">
-        <v>0.32643044200553584</v>
+        <v>0.33302080173822463</v>
       </c>
       <c r="C23" s="4">
         <f t="shared" si="0"/>
-        <v>46353122.764786087</v>
+        <v>47288953.846827894</v>
       </c>
       <c r="E23" s="4">
         <f t="shared" si="1"/>
@@ -1413,11 +1413,11 @@
         <v>22</v>
       </c>
       <c r="B24" s="3">
-        <v>0.34296152497092097</v>
+        <v>0.34078606641838294</v>
       </c>
       <c r="C24" s="4">
         <f t="shared" si="0"/>
-        <v>48700536.545870781</v>
+        <v>48391621.43141038</v>
       </c>
       <c r="E24" s="4">
         <f t="shared" si="1"/>
@@ -1429,11 +1429,11 @@
         <v>23</v>
       </c>
       <c r="B25" s="3">
-        <v>0.3453528608483149</v>
+        <v>0.34565145319866331</v>
       </c>
       <c r="C25" s="4">
         <f t="shared" si="0"/>
-        <v>49040106.240460716</v>
+        <v>49082506.35421019</v>
       </c>
       <c r="E25" s="4">
         <f t="shared" si="1"/>
@@ -1445,11 +1445,11 @@
         <v>24</v>
       </c>
       <c r="B26" s="3">
-        <v>0.37004276174482909</v>
+        <v>0.36402114934613722</v>
       </c>
       <c r="C26" s="4">
         <f t="shared" si="0"/>
-        <v>52546072.167765729</v>
+        <v>51691003.207151487</v>
       </c>
       <c r="E26" s="4">
         <f t="shared" si="1"/>
@@ -1461,11 +1461,11 @@
         <v>25</v>
       </c>
       <c r="B27" s="3">
-        <v>0.39272435790101479</v>
+        <v>0.38577853108457799</v>
       </c>
       <c r="C27" s="4">
         <f t="shared" si="0"/>
-        <v>55766858.821944103</v>
+        <v>54780551.414010078</v>
       </c>
       <c r="E27" s="4">
         <f t="shared" si="1"/>
@@ -1477,11 +1477,11 @@
         <v>26</v>
       </c>
       <c r="B28" s="3">
-        <v>0.40340547059461362</v>
+        <v>0.41724024949408756</v>
       </c>
       <c r="C28" s="4">
         <f t="shared" si="0"/>
-        <v>57283576.824435137</v>
+        <v>59248115.428160436</v>
       </c>
       <c r="E28" s="4">
         <f t="shared" si="1"/>
@@ -1493,11 +1493,11 @@
         <v>27</v>
       </c>
       <c r="B29" s="3">
-        <v>0.409773198998163</v>
+        <v>0.42837834616153569</v>
       </c>
       <c r="C29" s="4">
         <f t="shared" si="0"/>
-        <v>58187794.257739149</v>
+        <v>60829725.154938072</v>
       </c>
       <c r="E29" s="4">
         <f t="shared" si="1"/>
@@ -1509,11 +1509,11 @@
         <v>28</v>
       </c>
       <c r="B30" s="3">
-        <v>0.4385088884701433</v>
+        <v>0.43171235782888068</v>
       </c>
       <c r="C30" s="4">
         <f t="shared" si="0"/>
-        <v>62268262.162760347</v>
+        <v>61303154.811701059</v>
       </c>
       <c r="E30" s="4">
         <f t="shared" si="1"/>
@@ -1525,11 +1525,11 @@
         <v>29</v>
       </c>
       <c r="B31" s="3">
-        <v>0.44472863662132905</v>
+        <v>0.46518221262019155</v>
       </c>
       <c r="C31" s="4">
         <f t="shared" si="0"/>
-        <v>63151466.400228724</v>
+        <v>66055874.192067198</v>
       </c>
       <c r="E31" s="4">
         <f t="shared" si="1"/>
@@ -1541,11 +1541,11 @@
         <v>30</v>
       </c>
       <c r="B32" s="3">
-        <v>0.49648073777651436</v>
+        <v>0.49168193214591577</v>
       </c>
       <c r="C32" s="4">
         <f t="shared" si="0"/>
-        <v>70500264.764265046</v>
+        <v>69818834.364720032</v>
       </c>
       <c r="E32" s="4">
         <f t="shared" si="1"/>

</xml_diff>